<commit_message>
update ref in feedstock price data
</commit_message>
<xml_diff>
--- a/data/prices/feedstock_price_eia.xlsx
+++ b/data/prices/feedstock_price_eia.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\yale\Project-graphite\graphite_sus\data\price\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\qqisi\Susbiographite\data\prices\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56986FF7-19EC-4D8E-B8A4-8C47C84703D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E505969-706F-41CA-A1B0-38B56A646104}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="2" xr2:uid="{07F6B24B-2CD7-482F-9DC7-158F0658BBDC}"/>
   </bookViews>
@@ -428,9 +428,6 @@
     <t>MMBtu to short ton ref</t>
   </si>
   <si>
-    <t>https://www.epa.gov/system/files/documents/2022-10/Default%20Heat%20Content%20Ratios%20for%20Help%20and%20User%20Guide%20%281%29.pdf?utm_source=chatgpt.com</t>
-  </si>
-  <si>
     <t>minimum</t>
   </si>
   <si>
@@ -781,6 +778,9 @@
   </si>
   <si>
     <t>t</t>
+  </si>
+  <si>
+    <t>https://www.epa.gov/system/files/documents/2022-10/Default%20Heat%20Content%20Ratios%20for%20Help%20and%20User%20Guide%20%281%29.pdf</t>
   </si>
 </sst>
 </file>
@@ -1145,6 +1145,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1175,9 +1178,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1557,72 +1557,72 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="18" thickBot="1">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-      <c r="F1" s="26"/>
-      <c r="G1" s="26"/>
-      <c r="H1" s="26"/>
-      <c r="I1" s="26"/>
-      <c r="J1" s="26"/>
-      <c r="K1" s="26"/>
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="27"/>
+      <c r="G1" s="27"/>
+      <c r="H1" s="27"/>
+      <c r="I1" s="27"/>
+      <c r="J1" s="27"/>
+      <c r="K1" s="27"/>
       <c r="M1" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="2" spans="1:13" ht="15" thickBot="1">
-      <c r="A2" s="27" t="s">
+      <c r="A2" s="28" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="30" t="s">
+      <c r="B2" s="31" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="31"/>
-      <c r="D2" s="31"/>
-      <c r="E2" s="31"/>
-      <c r="F2" s="32"/>
-      <c r="G2" s="30" t="s">
+      <c r="C2" s="32"/>
+      <c r="D2" s="32"/>
+      <c r="E2" s="32"/>
+      <c r="F2" s="33"/>
+      <c r="G2" s="31" t="s">
         <v>3</v>
       </c>
-      <c r="H2" s="31"/>
-      <c r="I2" s="31"/>
-      <c r="J2" s="31"/>
-      <c r="K2" s="32"/>
+      <c r="H2" s="32"/>
+      <c r="I2" s="32"/>
+      <c r="J2" s="32"/>
+      <c r="K2" s="33"/>
       <c r="M2" s="10" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="3" spans="1:13" ht="15" thickBot="1">
-      <c r="A3" s="28"/>
+      <c r="A3" s="29"/>
       <c r="B3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="30" t="s">
+      <c r="C3" s="31" t="s">
         <v>5</v>
       </c>
-      <c r="D3" s="31"/>
-      <c r="E3" s="32"/>
-      <c r="F3" s="27" t="s">
+      <c r="D3" s="32"/>
+      <c r="E3" s="33"/>
+      <c r="F3" s="28" t="s">
         <v>6</v>
       </c>
       <c r="G3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="H3" s="30" t="s">
+      <c r="H3" s="31" t="s">
         <v>5</v>
       </c>
-      <c r="I3" s="31"/>
-      <c r="J3" s="32"/>
-      <c r="K3" s="27" t="s">
+      <c r="I3" s="32"/>
+      <c r="J3" s="33"/>
+      <c r="K3" s="28" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:13" ht="15" thickBot="1">
-      <c r="A4" s="28"/>
+      <c r="A4" s="29"/>
       <c r="B4" s="1" t="s">
         <v>7</v>
       </c>
@@ -1635,7 +1635,7 @@
       <c r="E4" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="F4" s="29"/>
+      <c r="F4" s="30"/>
       <c r="G4" s="1" t="s">
         <v>7</v>
       </c>
@@ -1648,24 +1648,24 @@
       <c r="J4" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="K4" s="29"/>
+      <c r="K4" s="30"/>
     </row>
     <row r="5" spans="1:13" ht="15" thickBot="1">
-      <c r="A5" s="29"/>
-      <c r="B5" s="33" t="s">
+      <c r="A5" s="30"/>
+      <c r="B5" s="34" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="34"/>
-      <c r="D5" s="34"/>
-      <c r="E5" s="34"/>
-      <c r="F5" s="35"/>
-      <c r="G5" s="33" t="s">
+      <c r="C5" s="35"/>
+      <c r="D5" s="35"/>
+      <c r="E5" s="35"/>
+      <c r="F5" s="36"/>
+      <c r="G5" s="34" t="s">
         <v>12</v>
       </c>
-      <c r="H5" s="34"/>
-      <c r="I5" s="34"/>
-      <c r="J5" s="34"/>
-      <c r="K5" s="35"/>
+      <c r="H5" s="35"/>
+      <c r="I5" s="35"/>
+      <c r="J5" s="35"/>
+      <c r="K5" s="36"/>
     </row>
     <row r="6" spans="1:13" ht="15" thickBot="1">
       <c r="A6" s="2" t="s">
@@ -3517,36 +3517,36 @@
   <sheetData>
     <row r="1" spans="1:9">
       <c r="A1" t="s">
+        <v>155</v>
+      </c>
+      <c r="B1" t="s">
         <v>156</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>157</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>158</v>
       </c>
-      <c r="D1" t="s">
-        <v>159</v>
-      </c>
       <c r="E1" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="F1" t="s">
+        <v>178</v>
+      </c>
+      <c r="H1" t="s">
         <v>179</v>
       </c>
-      <c r="H1" t="s">
-        <v>180</v>
-      </c>
       <c r="I1" s="10" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="2" spans="1:9">
       <c r="A2" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B2" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C2">
         <v>9.74</v>
@@ -3559,7 +3559,7 @@
         <v>1.1301767995029724E-2</v>
       </c>
       <c r="H2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="I2">
         <v>2025</v>
@@ -3567,10 +3567,10 @@
     </row>
     <row r="3" spans="1:9">
       <c r="A3" t="s">
+        <v>160</v>
+      </c>
+      <c r="B3" t="s">
         <v>161</v>
-      </c>
-      <c r="B3" t="s">
-        <v>162</v>
       </c>
       <c r="C3">
         <v>4.9400000000000004</v>
@@ -3583,7 +3583,7 @@
         <v>5.7350684890979517E-3</v>
       </c>
       <c r="H3" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="I3">
         <v>2022</v>
@@ -3591,10 +3591,10 @@
     </row>
     <row r="4" spans="1:9">
       <c r="A4" t="s">
+        <v>162</v>
+      </c>
+      <c r="B4" t="s">
         <v>163</v>
-      </c>
-      <c r="B4" t="s">
-        <v>164</v>
       </c>
       <c r="C4">
         <v>8.41</v>
@@ -3609,10 +3609,10 @@
     </row>
     <row r="5" spans="1:9">
       <c r="A5" t="s">
+        <v>164</v>
+      </c>
+      <c r="B5" t="s">
         <v>165</v>
-      </c>
-      <c r="B5" t="s">
-        <v>166</v>
       </c>
       <c r="C5">
         <v>10.84</v>
@@ -3627,10 +3627,10 @@
     </row>
     <row r="6" spans="1:9">
       <c r="A6" t="s">
+        <v>166</v>
+      </c>
+      <c r="B6" t="s">
         <v>167</v>
-      </c>
-      <c r="B6" t="s">
-        <v>168</v>
       </c>
       <c r="C6">
         <v>0.68</v>
@@ -3645,10 +3645,10 @@
     </row>
     <row r="7" spans="1:9">
       <c r="A7" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B7" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C7">
         <v>29</v>
@@ -3661,15 +3661,15 @@
         <v>3.3642227448892018E-2</v>
       </c>
       <c r="F7" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="8" spans="1:9">
       <c r="A8" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B8" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C8">
         <v>2.65</v>
@@ -3682,15 +3682,15 @@
         <v>3.0727339427827557E-3</v>
       </c>
       <c r="F8" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="9" spans="1:9">
       <c r="A9" t="s">
+        <v>170</v>
+      </c>
+      <c r="B9" t="s">
         <v>171</v>
-      </c>
-      <c r="B9" t="s">
-        <v>172</v>
       </c>
       <c r="C9">
         <v>2.96</v>
@@ -3703,12 +3703,12 @@
         <v>3.4305180320108849E-3</v>
       </c>
       <c r="F9" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="11" spans="1:9">
       <c r="A11" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="E11">
         <f>SUM(E2:E6)</f>
@@ -3717,12 +3717,12 @@
     </row>
     <row r="15" spans="1:9">
       <c r="A15" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="16" spans="1:9">
       <c r="A16" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B16">
         <f>MIN('2025_feed_price'!C2:C52)</f>
@@ -3731,7 +3731,7 @@
     </row>
     <row r="17" spans="1:2">
       <c r="A17" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B17">
         <f>MAX('2025_feed_price'!C2:C52)</f>
@@ -3762,16 +3762,16 @@
       <c r="A1" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="36">
+      <c r="B1" s="25">
         <v>2023</v>
       </c>
-      <c r="C1" s="36"/>
-      <c r="D1" s="36"/>
-      <c r="E1" s="36"/>
-      <c r="F1" s="36"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
       <c r="G1" s="24"/>
       <c r="L1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="2" spans="1:14" ht="49.8" thickBot="1">
@@ -3785,7 +3785,7 @@
         <v>69</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E2" s="8" t="s">
         <v>68</v>
@@ -3794,26 +3794,26 @@
         <v>70</v>
       </c>
       <c r="G2" s="11" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="H2" s="8" t="s">
         <v>68</v>
       </c>
       <c r="I2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="J2" s="11" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="K2" s="11" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="L2">
         <f>MIN(H3:H54)</f>
         <v>2.3318620070562426E-2</v>
       </c>
       <c r="M2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="N2" t="s">
         <v>73</v>
@@ -3853,10 +3853,10 @@
         <v>2025</v>
       </c>
       <c r="J3" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="K3" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="L3">
         <f>MAX(H3:H54)</f>
@@ -3900,17 +3900,17 @@
         <v>2025</v>
       </c>
       <c r="J4" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="K4" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="L4">
         <f>H54</f>
         <v>6.1784377964738062E-2</v>
       </c>
       <c r="M4" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="N4" t="s">
         <v>74</v>
@@ -3950,13 +3950,13 @@
         <v>2025</v>
       </c>
       <c r="J5" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="M5" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="N5" s="10" t="s">
-        <v>76</v>
+        <v>192</v>
       </c>
     </row>
     <row r="6" spans="1:14" ht="15" thickBot="1">
@@ -3993,13 +3993,13 @@
         <v>2025</v>
       </c>
       <c r="J6" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="L6" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="M6" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="7" spans="1:14" ht="15" thickBot="1">
@@ -4036,17 +4036,17 @@
         <v>2025</v>
       </c>
       <c r="J7" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="K7" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="L7">
         <f>MIN(D3:D54)</f>
         <v>20.451599999999999</v>
       </c>
       <c r="M7" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="8" spans="1:14" ht="15" thickBot="1">
@@ -4083,17 +4083,17 @@
         <v>2025</v>
       </c>
       <c r="J8" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="K8" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="L8">
         <f>MAX(D3:D54)</f>
         <v>60.306000000000004</v>
       </c>
       <c r="M8" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="9" spans="1:14" ht="15" thickBot="1">
@@ -4130,10 +4130,10 @@
         <v>2025</v>
       </c>
       <c r="J9" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="M9" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="10" spans="1:14" ht="15" thickBot="1">
@@ -4170,10 +4170,10 @@
         <v>2025</v>
       </c>
       <c r="J10" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="M10" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="11" spans="1:14" ht="15" thickBot="1">
@@ -4210,10 +4210,10 @@
         <v>2025</v>
       </c>
       <c r="J11" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="M11" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="12" spans="1:14" ht="15" thickBot="1">
@@ -4250,10 +4250,10 @@
         <v>2025</v>
       </c>
       <c r="J12" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="M12" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="13" spans="1:14" ht="15" thickBot="1">
@@ -4290,10 +4290,10 @@
         <v>2025</v>
       </c>
       <c r="J13" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="M13" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="14" spans="1:14" ht="15" thickBot="1">
@@ -4330,10 +4330,10 @@
         <v>2025</v>
       </c>
       <c r="J14" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="M14" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="15" spans="1:14" ht="15" thickBot="1">
@@ -4370,10 +4370,10 @@
         <v>2025</v>
       </c>
       <c r="J15" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="M15" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="16" spans="1:14" ht="15" thickBot="1">
@@ -4410,10 +4410,10 @@
         <v>2025</v>
       </c>
       <c r="J16" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="M16" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="17" spans="1:13" ht="15" thickBot="1">
@@ -4450,10 +4450,10 @@
         <v>2025</v>
       </c>
       <c r="J17" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="M17" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="18" spans="1:13" ht="15" thickBot="1">
@@ -4490,10 +4490,10 @@
         <v>2025</v>
       </c>
       <c r="J18" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="M18" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="19" spans="1:13" ht="15" thickBot="1">
@@ -4530,10 +4530,10 @@
         <v>2025</v>
       </c>
       <c r="J19" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="M19" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="20" spans="1:13" ht="15" thickBot="1">
@@ -4570,10 +4570,10 @@
         <v>2025</v>
       </c>
       <c r="J20" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="M20" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="21" spans="1:13" ht="15" thickBot="1">
@@ -4610,10 +4610,10 @@
         <v>2025</v>
       </c>
       <c r="J21" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="M21" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="22" spans="1:13" ht="15" thickBot="1">
@@ -4650,10 +4650,10 @@
         <v>2025</v>
       </c>
       <c r="J22" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="M22" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="23" spans="1:13" ht="15" thickBot="1">
@@ -4690,10 +4690,10 @@
         <v>2025</v>
       </c>
       <c r="J23" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="M23" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="24" spans="1:13" ht="15" thickBot="1">
@@ -4730,10 +4730,10 @@
         <v>2025</v>
       </c>
       <c r="J24" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="M24" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="25" spans="1:13" ht="15" thickBot="1">
@@ -4770,10 +4770,10 @@
         <v>2025</v>
       </c>
       <c r="J25" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="M25" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="26" spans="1:13" ht="15" thickBot="1">
@@ -4810,10 +4810,10 @@
         <v>2025</v>
       </c>
       <c r="J26" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="M26" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="27" spans="1:13" ht="15" thickBot="1">
@@ -4850,10 +4850,10 @@
         <v>2025</v>
       </c>
       <c r="J27" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="M27" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="28" spans="1:13" ht="15" thickBot="1">
@@ -4890,10 +4890,10 @@
         <v>2025</v>
       </c>
       <c r="J28" t="s">
+        <v>127</v>
+      </c>
+      <c r="M28" t="s">
         <v>128</v>
-      </c>
-      <c r="M28" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="29" spans="1:13" ht="15" thickBot="1">
@@ -4930,10 +4930,10 @@
         <v>2025</v>
       </c>
       <c r="J29" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="M29" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="30" spans="1:13" ht="15" thickBot="1">
@@ -4970,10 +4970,10 @@
         <v>2025</v>
       </c>
       <c r="J30" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="M30" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="31" spans="1:13" ht="15" thickBot="1">
@@ -5010,10 +5010,10 @@
         <v>2025</v>
       </c>
       <c r="J31" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="M31" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="32" spans="1:13" ht="15" thickBot="1">
@@ -5050,10 +5050,10 @@
         <v>2025</v>
       </c>
       <c r="J32" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="M32" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="33" spans="1:13" ht="15" thickBot="1">
@@ -5090,10 +5090,10 @@
         <v>2025</v>
       </c>
       <c r="J33" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="M33" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="34" spans="1:13" ht="15" thickBot="1">
@@ -5130,10 +5130,10 @@
         <v>2025</v>
       </c>
       <c r="J34" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="M34" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="35" spans="1:13" ht="15" thickBot="1">
@@ -5170,10 +5170,10 @@
         <v>2025</v>
       </c>
       <c r="J35" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="M35" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="36" spans="1:13" ht="15" thickBot="1">
@@ -5210,10 +5210,10 @@
         <v>2025</v>
       </c>
       <c r="J36" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="M36" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="37" spans="1:13" ht="15" thickBot="1">
@@ -5250,10 +5250,10 @@
         <v>2025</v>
       </c>
       <c r="J37" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="M37" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="38" spans="1:13" ht="15" thickBot="1">
@@ -5290,10 +5290,10 @@
         <v>2025</v>
       </c>
       <c r="J38" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="M38" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="39" spans="1:13" ht="15" thickBot="1">
@@ -5330,10 +5330,10 @@
         <v>2025</v>
       </c>
       <c r="J39" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="M39" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="40" spans="1:13" ht="15" thickBot="1">
@@ -5370,10 +5370,10 @@
         <v>2025</v>
       </c>
       <c r="J40" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="M40" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="41" spans="1:13" ht="15" thickBot="1">
@@ -5410,10 +5410,10 @@
         <v>2025</v>
       </c>
       <c r="J41" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="M41" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="42" spans="1:13" ht="15" thickBot="1">
@@ -5450,10 +5450,10 @@
         <v>2025</v>
       </c>
       <c r="J42" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="M42" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="43" spans="1:13" ht="15" thickBot="1">
@@ -5490,10 +5490,10 @@
         <v>2025</v>
       </c>
       <c r="J43" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="M43" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="44" spans="1:13" ht="15" thickBot="1">
@@ -5530,10 +5530,10 @@
         <v>2025</v>
       </c>
       <c r="J44" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="M44" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="45" spans="1:13" ht="15" thickBot="1">
@@ -5570,10 +5570,10 @@
         <v>2025</v>
       </c>
       <c r="J45" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M45" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="46" spans="1:13" ht="15" thickBot="1">
@@ -5610,10 +5610,10 @@
         <v>2025</v>
       </c>
       <c r="J46" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="M46" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="47" spans="1:13" ht="15" thickBot="1">
@@ -5650,10 +5650,10 @@
         <v>2025</v>
       </c>
       <c r="J47" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="M47" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="48" spans="1:13" ht="15" thickBot="1">
@@ -5690,10 +5690,10 @@
         <v>2025</v>
       </c>
       <c r="J48" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="M48" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="49" spans="1:13" ht="15" thickBot="1">
@@ -5730,10 +5730,10 @@
         <v>2025</v>
       </c>
       <c r="J49" t="s">
+        <v>148</v>
+      </c>
+      <c r="M49" t="s">
         <v>149</v>
-      </c>
-      <c r="M49" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="50" spans="1:13" ht="15" thickBot="1">
@@ -5770,10 +5770,10 @@
         <v>2025</v>
       </c>
       <c r="J50" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="M50" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="51" spans="1:13" ht="15" thickBot="1">
@@ -5810,10 +5810,10 @@
         <v>2025</v>
       </c>
       <c r="J51" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="M51" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="52" spans="1:13" ht="15" thickBot="1">
@@ -5850,10 +5850,10 @@
         <v>2025</v>
       </c>
       <c r="J52" t="s">
+        <v>151</v>
+      </c>
+      <c r="M52" t="s">
         <v>152</v>
-      </c>
-      <c r="M52" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="53" spans="1:13" ht="15" thickBot="1">
@@ -5890,10 +5890,10 @@
         <v>2025</v>
       </c>
       <c r="J53" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="M53" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="54" spans="1:13" ht="15" thickBot="1">
@@ -5956,13 +5956,13 @@
         <v>1</v>
       </c>
       <c r="B1" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C1" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="D1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="2" spans="1:4">
@@ -5977,7 +5977,7 @@
         <v>0.10632507824091753</v>
       </c>
       <c r="D2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -5992,7 +5992,7 @@
         <v>7.0450278132359948E-2</v>
       </c>
       <c r="D3" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -6007,7 +6007,7 @@
         <v>0.10014664044444371</v>
       </c>
       <c r="D4" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -6022,7 +6022,7 @@
         <v>0.10512925157063227</v>
       </c>
       <c r="D5" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -6037,7 +6037,7 @@
         <v>0.10293690267510933</v>
       </c>
       <c r="D6" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -6052,7 +6052,7 @@
         <v>0.10094385822463389</v>
       </c>
       <c r="D7" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -6067,7 +6067,7 @@
         <v>9.4566115983112542E-2</v>
       </c>
       <c r="D8" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -6082,7 +6082,7 @@
         <v>6.347462255569597E-2</v>
       </c>
       <c r="D9" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -6097,7 +6097,7 @@
         <v>9.2971680422732211E-2</v>
       </c>
       <c r="D10" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -6112,7 +6112,7 @@
         <v>9.1377244862351867E-2</v>
       </c>
       <c r="D11" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -6127,7 +6127,7 @@
         <v>0.10592646935082245</v>
       </c>
       <c r="D12" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -6142,7 +6142,7 @@
         <v>9.9548727109301099E-2</v>
       </c>
       <c r="D13" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -6157,7 +6157,7 @@
         <v>0.10612577379586999</v>
       </c>
       <c r="D14" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -6172,7 +6172,7 @@
         <v>8.6394633736163323E-2</v>
       </c>
       <c r="D15" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -6187,7 +6187,7 @@
         <v>9.2174462642542032E-2</v>
       </c>
       <c r="D16" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="17" spans="1:4">
@@ -6202,7 +6202,7 @@
         <v>9.2971680422732211E-2</v>
       </c>
       <c r="D17" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="18" spans="1:4">
@@ -6217,7 +6217,7 @@
         <v>6.4271840335886149E-2</v>
       </c>
       <c r="D18" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="19" spans="1:4">
@@ -6232,7 +6232,7 @@
         <v>0.10094385822463389</v>
       </c>
       <c r="D19" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="20" spans="1:4">
@@ -6247,7 +6247,7 @@
         <v>0.10293690267510933</v>
       </c>
       <c r="D20" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="21" spans="1:4">
@@ -6262,7 +6262,7 @@
         <v>0.10552786046072735</v>
       </c>
       <c r="D21" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="22" spans="1:4">
@@ -6277,7 +6277,7 @@
         <v>9.2971680422732211E-2</v>
       </c>
       <c r="D22" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="23" spans="1:4">
@@ -6292,7 +6292,7 @@
         <v>8.8786287076733819E-2</v>
       </c>
       <c r="D23" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="24" spans="1:4">
@@ -6307,7 +6307,7 @@
         <v>9.915011821920601E-2</v>
       </c>
       <c r="D24" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="25" spans="1:4">
@@ -6322,7 +6322,7 @@
         <v>0.10532855601567981</v>
       </c>
       <c r="D25" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="26" spans="1:4">
@@ -6337,7 +6337,7 @@
         <v>0.10572716490577491</v>
       </c>
       <c r="D26" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="27" spans="1:4">
@@ -6352,7 +6352,7 @@
         <v>9.4366811538065004E-2</v>
       </c>
       <c r="D27" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="28" spans="1:4">
@@ -6367,7 +6367,7 @@
         <v>9.5961247098445335E-2</v>
       </c>
       <c r="D28" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="29" spans="1:4">
@@ -6382,7 +6382,7 @@
         <v>6.6663493676456645E-2</v>
       </c>
       <c r="D29" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="30" spans="1:4">
@@ -6397,7 +6397,7 @@
         <v>0.10014664044444371</v>
       </c>
       <c r="D30" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="31" spans="1:4">
@@ -6412,7 +6412,7 @@
         <v>7.3639149253120623E-2</v>
       </c>
       <c r="D31" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="32" spans="1:4">
@@ -6427,7 +6427,7 @@
         <v>8.4002980395592813E-2</v>
       </c>
       <c r="D32" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="33" spans="1:4">
@@ -6442,7 +6442,7 @@
         <v>0.10891603602653557</v>
       </c>
       <c r="D33" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="34" spans="1:4">
@@ -6457,7 +6457,7 @@
         <v>9.4964724873207632E-2</v>
       </c>
       <c r="D34" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="35" spans="1:4">
@@ -6472,7 +6472,7 @@
         <v>0.10572716490577491</v>
       </c>
       <c r="D35" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="36" spans="1:4">
@@ -6487,7 +6487,7 @@
         <v>9.0580027082161702E-2</v>
       </c>
       <c r="D36" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="37" spans="1:4">
@@ -6502,7 +6502,7 @@
         <v>8.6195329291115785E-2</v>
       </c>
       <c r="D37" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="38" spans="1:4">
@@ -6517,7 +6517,7 @@
         <v>9.2772375977684673E-2</v>
       </c>
       <c r="D38" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="39" spans="1:4">
@@ -6532,7 +6532,7 @@
         <v>0.10353481601025194</v>
       </c>
       <c r="D39" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="40" spans="1:4">
@@ -6547,7 +6547,7 @@
         <v>8.4800198175782993E-2</v>
       </c>
       <c r="D40" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="41" spans="1:4">
@@ -6562,7 +6562,7 @@
         <v>9.1775853752446956E-2</v>
       </c>
       <c r="D41" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="42" spans="1:4">
@@ -6577,7 +6577,7 @@
         <v>0.10552786046072735</v>
       </c>
       <c r="D42" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="43" spans="1:4">
@@ -6592,7 +6592,7 @@
         <v>0.10453133823548966</v>
       </c>
       <c r="D43" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="44" spans="1:4">
@@ -6607,7 +6607,7 @@
         <v>0.10114316266968144</v>
       </c>
       <c r="D44" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="45" spans="1:4">
@@ -6622,7 +6622,7 @@
         <v>9.2971680422732211E-2</v>
       </c>
       <c r="D45" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="46" spans="1:4">
@@ -6637,7 +6637,7 @@
         <v>0.10213968489491913</v>
       </c>
       <c r="D46" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="47" spans="1:4">
@@ -6652,7 +6652,7 @@
         <v>0.10094385822463389</v>
       </c>
       <c r="D47" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="48" spans="1:4">
@@ -6667,7 +6667,7 @@
         <v>0.10512925157063227</v>
       </c>
       <c r="D48" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="49" spans="1:4">
@@ -6682,7 +6682,7 @@
         <v>0.10433203379044212</v>
       </c>
       <c r="D49" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="50" spans="1:4">
@@ -6697,7 +6697,7 @@
         <v>8.9982113747019088E-2</v>
       </c>
       <c r="D50" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="51" spans="1:4">
@@ -6712,7 +6712,7 @@
         <v>9.915011821920601E-2</v>
       </c>
       <c r="D51" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="52" spans="1:4">
@@ -6727,7 +6727,7 @@
         <v>9.875150932911092E-2</v>
       </c>
       <c r="D52" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
   </sheetData>
@@ -6745,33 +6745,33 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="15" thickBot="1">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="28" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="30" t="s">
+      <c r="B1" s="31" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
-      <c r="E1" s="31"/>
-      <c r="F1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="33"/>
     </row>
     <row r="2" spans="1:9" ht="15" thickBot="1">
-      <c r="A2" s="28"/>
+      <c r="A2" s="29"/>
       <c r="B2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="30" t="s">
+      <c r="C2" s="31" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="31"/>
-      <c r="E2" s="32"/>
-      <c r="F2" s="27" t="s">
+      <c r="D2" s="32"/>
+      <c r="E2" s="33"/>
+      <c r="F2" s="28" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="40.200000000000003" thickBot="1">
-      <c r="A3" s="28"/>
+      <c r="A3" s="29"/>
       <c r="B3" s="1" t="s">
         <v>7</v>
       </c>
@@ -6784,26 +6784,26 @@
       <c r="E3" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="F3" s="29"/>
+      <c r="F3" s="30"/>
       <c r="G3" s="8" t="s">
+        <v>187</v>
+      </c>
+      <c r="H3" s="8" t="s">
         <v>188</v>
       </c>
-      <c r="H3" s="8" t="s">
+      <c r="I3" s="8" t="s">
         <v>189</v>
       </c>
-      <c r="I3" s="8" t="s">
-        <v>190</v>
-      </c>
     </row>
     <row r="4" spans="1:9" ht="15" thickBot="1">
-      <c r="A4" s="29"/>
-      <c r="B4" s="33" t="s">
+      <c r="A4" s="30"/>
+      <c r="B4" s="34" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="34"/>
-      <c r="D4" s="34"/>
-      <c r="E4" s="34"/>
-      <c r="F4" s="35"/>
+      <c r="C4" s="35"/>
+      <c r="D4" s="35"/>
+      <c r="E4" s="35"/>
+      <c r="F4" s="36"/>
     </row>
     <row r="5" spans="1:9" ht="15" thickBot="1">
       <c r="A5" s="2" t="s">
@@ -8282,38 +8282,38 @@
     </row>
     <row r="2" spans="1:18" ht="18">
       <c r="B2" s="14" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G2" s="13"/>
       <c r="I2" s="14" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="O2" s="13"/>
       <c r="Q2" s="15" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="R2" s="16"/>
     </row>
     <row r="3" spans="1:18">
       <c r="B3" t="s">
+        <v>84</v>
+      </c>
+      <c r="C3" t="s">
         <v>85</v>
-      </c>
-      <c r="C3" t="s">
-        <v>86</v>
       </c>
       <c r="G3" s="13"/>
       <c r="I3" t="s">
+        <v>86</v>
+      </c>
+      <c r="J3" s="10" t="s">
         <v>87</v>
-      </c>
-      <c r="J3" s="10" t="s">
-        <v>88</v>
       </c>
       <c r="O3" s="13"/>
       <c r="Q3" s="16" t="s">
+        <v>88</v>
+      </c>
+      <c r="R3" s="16" t="s">
         <v>89</v>
-      </c>
-      <c r="R3" s="16" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="4" spans="1:18">
@@ -8321,17 +8321,17 @@
       <c r="K4" s="10"/>
       <c r="O4" s="13"/>
       <c r="Q4" s="17" t="s">
+        <v>90</v>
+      </c>
+      <c r="R4" s="16" t="s">
         <v>91</v>
-      </c>
-      <c r="R4" s="16" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="5" spans="1:18">
       <c r="G5" s="13"/>
       <c r="O5" s="13"/>
       <c r="Q5" s="16" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="R5" s="16"/>
     </row>
@@ -8339,7 +8339,7 @@
       <c r="G6" s="13"/>
       <c r="O6" s="13"/>
       <c r="Q6" s="16" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="R6" s="16"/>
     </row>
@@ -8348,7 +8348,7 @@
       <c r="O7" s="13"/>
       <c r="Q7" s="16"/>
       <c r="R7" s="17" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="8" spans="1:18">
@@ -8370,34 +8370,34 @@
     </row>
     <row r="12" spans="1:18">
       <c r="A12" s="18" t="s">
+        <v>95</v>
+      </c>
+      <c r="B12" s="18" t="s">
         <v>96</v>
       </c>
-      <c r="B12" s="18" t="s">
+      <c r="C12" s="18" t="s">
         <v>97</v>
-      </c>
-      <c r="C12" s="18" t="s">
-        <v>98</v>
       </c>
       <c r="G12" s="13"/>
       <c r="H12" s="19"/>
       <c r="I12" s="18" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="J12" s="18" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="O12" s="13"/>
       <c r="P12" s="19"/>
       <c r="Q12" s="18" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="R12" s="18" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="13" spans="1:18">
       <c r="A13" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B13" s="19">
         <v>1990</v>
@@ -8407,7 +8407,7 @@
       </c>
       <c r="G13" s="13"/>
       <c r="H13" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I13" s="19">
         <v>1980</v>
@@ -8417,7 +8417,7 @@
       </c>
       <c r="O13" s="13"/>
       <c r="P13" s="19" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="Q13" s="19">
         <v>1980</v>
@@ -8428,7 +8428,7 @@
     </row>
     <row r="14" spans="1:18">
       <c r="A14" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B14" s="19">
         <v>1991</v>
@@ -8438,7 +8438,7 @@
       </c>
       <c r="G14" s="13"/>
       <c r="H14" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I14" s="19">
         <v>1981</v>
@@ -8448,7 +8448,7 @@
       </c>
       <c r="O14" s="13"/>
       <c r="P14" s="19" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="Q14" s="19">
         <v>1981</v>
@@ -8459,7 +8459,7 @@
     </row>
     <row r="15" spans="1:18">
       <c r="A15" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B15" s="19">
         <v>1992</v>
@@ -8469,7 +8469,7 @@
       </c>
       <c r="G15" s="13"/>
       <c r="H15" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I15" s="19">
         <v>1982</v>
@@ -8479,7 +8479,7 @@
       </c>
       <c r="O15" s="13"/>
       <c r="P15" s="19" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="Q15" s="19">
         <v>1982</v>
@@ -8490,7 +8490,7 @@
     </row>
     <row r="16" spans="1:18">
       <c r="A16" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B16" s="19">
         <v>1993</v>
@@ -8500,7 +8500,7 @@
       </c>
       <c r="G16" s="13"/>
       <c r="H16" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I16" s="19">
         <v>1983</v>
@@ -8510,7 +8510,7 @@
       </c>
       <c r="O16" s="13"/>
       <c r="P16" s="19" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="Q16" s="19">
         <v>1983</v>
@@ -8521,7 +8521,7 @@
     </row>
     <row r="17" spans="1:18">
       <c r="A17" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B17" s="19">
         <v>1994</v>
@@ -8531,7 +8531,7 @@
       </c>
       <c r="G17" s="13"/>
       <c r="H17" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I17" s="19">
         <v>1984</v>
@@ -8541,7 +8541,7 @@
       </c>
       <c r="O17" s="13"/>
       <c r="P17" s="19" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="Q17" s="19">
         <v>1984</v>
@@ -8552,7 +8552,7 @@
     </row>
     <row r="18" spans="1:18">
       <c r="A18" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B18" s="19">
         <v>1995</v>
@@ -8562,7 +8562,7 @@
       </c>
       <c r="G18" s="13"/>
       <c r="H18" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I18" s="19">
         <v>1985</v>
@@ -8572,7 +8572,7 @@
       </c>
       <c r="O18" s="13"/>
       <c r="P18" s="19" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="Q18" s="19">
         <v>1985</v>
@@ -8583,7 +8583,7 @@
     </row>
     <row r="19" spans="1:18">
       <c r="A19" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B19" s="19">
         <v>1996</v>
@@ -8593,7 +8593,7 @@
       </c>
       <c r="G19" s="13"/>
       <c r="H19" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I19" s="19">
         <v>1986</v>
@@ -8603,7 +8603,7 @@
       </c>
       <c r="O19" s="13"/>
       <c r="P19" s="19" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="Q19" s="19">
         <v>1986</v>
@@ -8614,7 +8614,7 @@
     </row>
     <row r="20" spans="1:18">
       <c r="A20" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B20" s="19">
         <v>1997</v>
@@ -8624,7 +8624,7 @@
       </c>
       <c r="G20" s="13"/>
       <c r="H20" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I20" s="19">
         <v>1987</v>
@@ -8634,7 +8634,7 @@
       </c>
       <c r="O20" s="13"/>
       <c r="P20" s="19" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="Q20" s="19">
         <v>1987</v>
@@ -8645,7 +8645,7 @@
     </row>
     <row r="21" spans="1:18">
       <c r="A21" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B21" s="19">
         <v>1998</v>
@@ -8655,7 +8655,7 @@
       </c>
       <c r="G21" s="13"/>
       <c r="H21" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I21" s="19">
         <v>1988</v>
@@ -8665,7 +8665,7 @@
       </c>
       <c r="O21" s="13"/>
       <c r="P21" s="19" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="Q21" s="19">
         <v>1988</v>
@@ -8676,7 +8676,7 @@
     </row>
     <row r="22" spans="1:18">
       <c r="A22" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B22" s="19">
         <v>1999</v>
@@ -8686,7 +8686,7 @@
       </c>
       <c r="G22" s="13"/>
       <c r="H22" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I22" s="19">
         <v>1989</v>
@@ -8696,7 +8696,7 @@
       </c>
       <c r="O22" s="13"/>
       <c r="P22" s="19" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="Q22" s="19">
         <v>1989</v>
@@ -8707,7 +8707,7 @@
     </row>
     <row r="23" spans="1:18">
       <c r="A23" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B23" s="19">
         <v>2000</v>
@@ -8717,7 +8717,7 @@
       </c>
       <c r="G23" s="13"/>
       <c r="H23" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I23" s="19">
         <v>1990</v>
@@ -8727,7 +8727,7 @@
       </c>
       <c r="O23" s="13"/>
       <c r="P23" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="Q23" s="19">
         <v>1990</v>
@@ -8738,7 +8738,7 @@
     </row>
     <row r="24" spans="1:18">
       <c r="A24" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B24" s="19">
         <v>2001</v>
@@ -8748,7 +8748,7 @@
       </c>
       <c r="G24" s="13"/>
       <c r="H24" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I24" s="19">
         <v>1991</v>
@@ -8758,7 +8758,7 @@
       </c>
       <c r="O24" s="13"/>
       <c r="P24" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="Q24" s="19">
         <v>1991</v>
@@ -8769,7 +8769,7 @@
     </row>
     <row r="25" spans="1:18">
       <c r="A25" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B25" s="19">
         <v>2002</v>
@@ -8779,7 +8779,7 @@
       </c>
       <c r="G25" s="13"/>
       <c r="H25" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I25" s="19">
         <v>1992</v>
@@ -8789,7 +8789,7 @@
       </c>
       <c r="O25" s="13"/>
       <c r="P25" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="Q25" s="19">
         <v>1992</v>
@@ -8800,7 +8800,7 @@
     </row>
     <row r="26" spans="1:18">
       <c r="A26" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B26" s="19">
         <v>2003</v>
@@ -8810,7 +8810,7 @@
       </c>
       <c r="G26" s="13"/>
       <c r="H26" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I26" s="19">
         <v>1993</v>
@@ -8820,7 +8820,7 @@
       </c>
       <c r="O26" s="13"/>
       <c r="P26" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="Q26" s="19">
         <v>1993</v>
@@ -8831,7 +8831,7 @@
     </row>
     <row r="27" spans="1:18">
       <c r="A27" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B27" s="19">
         <v>2004</v>
@@ -8841,7 +8841,7 @@
       </c>
       <c r="G27" s="13"/>
       <c r="H27" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I27" s="19">
         <v>1994</v>
@@ -8851,7 +8851,7 @@
       </c>
       <c r="O27" s="13"/>
       <c r="P27" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="Q27" s="19">
         <v>1994</v>
@@ -8862,7 +8862,7 @@
     </row>
     <row r="28" spans="1:18">
       <c r="A28" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B28" s="19">
         <v>2005</v>
@@ -8872,7 +8872,7 @@
       </c>
       <c r="G28" s="13"/>
       <c r="H28" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I28" s="19">
         <v>1995</v>
@@ -8882,7 +8882,7 @@
       </c>
       <c r="O28" s="13"/>
       <c r="P28" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="Q28" s="19">
         <v>1995</v>
@@ -8893,7 +8893,7 @@
     </row>
     <row r="29" spans="1:18">
       <c r="A29" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B29" s="19">
         <v>2006</v>
@@ -8903,7 +8903,7 @@
       </c>
       <c r="G29" s="13"/>
       <c r="H29" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I29" s="19">
         <v>1996</v>
@@ -8913,7 +8913,7 @@
       </c>
       <c r="O29" s="13"/>
       <c r="P29" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="Q29" s="19">
         <v>1996</v>
@@ -8924,7 +8924,7 @@
     </row>
     <row r="30" spans="1:18">
       <c r="A30" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B30" s="19">
         <v>2007</v>
@@ -8934,7 +8934,7 @@
       </c>
       <c r="G30" s="13"/>
       <c r="H30" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I30" s="19">
         <v>1997</v>
@@ -8944,7 +8944,7 @@
       </c>
       <c r="O30" s="13"/>
       <c r="P30" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="Q30" s="19">
         <v>1997</v>
@@ -8955,7 +8955,7 @@
     </row>
     <row r="31" spans="1:18">
       <c r="A31" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B31" s="19">
         <v>2008</v>
@@ -8965,7 +8965,7 @@
       </c>
       <c r="G31" s="13"/>
       <c r="H31" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I31" s="19">
         <v>1998</v>
@@ -8975,7 +8975,7 @@
       </c>
       <c r="O31" s="13"/>
       <c r="P31" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="Q31" s="19">
         <v>1998</v>
@@ -8986,7 +8986,7 @@
     </row>
     <row r="32" spans="1:18">
       <c r="A32" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B32" s="19">
         <v>2009</v>
@@ -8996,7 +8996,7 @@
       </c>
       <c r="G32" s="13"/>
       <c r="H32" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I32" s="19">
         <v>1999</v>
@@ -9006,7 +9006,7 @@
       </c>
       <c r="O32" s="13"/>
       <c r="P32" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="Q32" s="19">
         <v>1999</v>
@@ -9017,7 +9017,7 @@
     </row>
     <row r="33" spans="1:18">
       <c r="A33" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B33" s="19">
         <v>2010</v>
@@ -9027,7 +9027,7 @@
       </c>
       <c r="G33" s="13"/>
       <c r="H33" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I33" s="19">
         <v>2000</v>
@@ -9037,7 +9037,7 @@
       </c>
       <c r="O33" s="13"/>
       <c r="P33" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="Q33" s="19">
         <v>2000</v>
@@ -9048,7 +9048,7 @@
     </row>
     <row r="34" spans="1:18">
       <c r="A34" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B34" s="19">
         <v>2011</v>
@@ -9058,7 +9058,7 @@
       </c>
       <c r="G34" s="13"/>
       <c r="H34" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I34" s="19">
         <v>2001</v>
@@ -9068,7 +9068,7 @@
       </c>
       <c r="O34" s="13"/>
       <c r="P34" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="Q34" s="19">
         <v>2001</v>
@@ -9079,7 +9079,7 @@
     </row>
     <row r="35" spans="1:18">
       <c r="A35" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B35" s="19">
         <v>2012</v>
@@ -9089,7 +9089,7 @@
       </c>
       <c r="G35" s="13"/>
       <c r="H35" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I35" s="19">
         <v>2002</v>
@@ -9099,7 +9099,7 @@
       </c>
       <c r="O35" s="13"/>
       <c r="P35" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="Q35" s="19">
         <v>2002</v>
@@ -9110,7 +9110,7 @@
     </row>
     <row r="36" spans="1:18">
       <c r="A36" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B36" s="19">
         <v>2013</v>
@@ -9120,7 +9120,7 @@
       </c>
       <c r="G36" s="13"/>
       <c r="H36" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I36" s="19">
         <v>2003</v>
@@ -9130,7 +9130,7 @@
       </c>
       <c r="O36" s="13"/>
       <c r="P36" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="Q36" s="19">
         <v>2003</v>
@@ -9141,7 +9141,7 @@
     </row>
     <row r="37" spans="1:18">
       <c r="A37" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B37" s="19">
         <v>2014</v>
@@ -9151,7 +9151,7 @@
       </c>
       <c r="G37" s="13"/>
       <c r="H37" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I37" s="19">
         <v>2004</v>
@@ -9161,7 +9161,7 @@
       </c>
       <c r="O37" s="13"/>
       <c r="P37" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="Q37" s="19">
         <v>2004</v>
@@ -9172,7 +9172,7 @@
     </row>
     <row r="38" spans="1:18">
       <c r="A38" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B38" s="19">
         <v>2015</v>
@@ -9182,7 +9182,7 @@
       </c>
       <c r="G38" s="13"/>
       <c r="H38" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I38" s="19">
         <v>2005</v>
@@ -9192,7 +9192,7 @@
       </c>
       <c r="O38" s="13"/>
       <c r="P38" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="Q38" s="19">
         <v>2005</v>
@@ -9203,7 +9203,7 @@
     </row>
     <row r="39" spans="1:18">
       <c r="A39" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B39" s="19">
         <v>2016</v>
@@ -9213,7 +9213,7 @@
       </c>
       <c r="G39" s="13"/>
       <c r="H39" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I39" s="19">
         <v>2006</v>
@@ -9223,7 +9223,7 @@
       </c>
       <c r="O39" s="13"/>
       <c r="P39" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="Q39" s="19">
         <v>2006</v>
@@ -9234,7 +9234,7 @@
     </row>
     <row r="40" spans="1:18">
       <c r="A40" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B40" s="19">
         <v>2017</v>
@@ -9244,7 +9244,7 @@
       </c>
       <c r="G40" s="13"/>
       <c r="H40" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I40" s="19">
         <v>2007</v>
@@ -9254,7 +9254,7 @@
       </c>
       <c r="O40" s="13"/>
       <c r="P40" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="Q40" s="19">
         <v>2007</v>
@@ -9265,7 +9265,7 @@
     </row>
     <row r="41" spans="1:18">
       <c r="A41" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B41" s="19">
         <v>2018</v>
@@ -9275,7 +9275,7 @@
       </c>
       <c r="G41" s="13"/>
       <c r="H41" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I41" s="19">
         <v>2008</v>
@@ -9285,7 +9285,7 @@
       </c>
       <c r="O41" s="13"/>
       <c r="P41" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="Q41" s="19">
         <v>2008</v>
@@ -9296,7 +9296,7 @@
     </row>
     <row r="42" spans="1:18">
       <c r="A42" s="19" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B42" s="19">
         <v>2019</v>
@@ -9306,7 +9306,7 @@
       </c>
       <c r="G42" s="13"/>
       <c r="H42" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I42" s="19">
         <v>2009</v>
@@ -9316,7 +9316,7 @@
       </c>
       <c r="O42" s="13"/>
       <c r="P42" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="Q42" s="19">
         <v>2009</v>
@@ -9327,7 +9327,7 @@
     </row>
     <row r="43" spans="1:18">
       <c r="A43" s="19" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B43" s="19">
         <v>2020</v>
@@ -9337,7 +9337,7 @@
       </c>
       <c r="G43" s="13"/>
       <c r="H43" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I43" s="19">
         <v>2010</v>
@@ -9347,7 +9347,7 @@
       </c>
       <c r="O43" s="13"/>
       <c r="P43" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="Q43" s="19">
         <v>2010</v>
@@ -9358,7 +9358,7 @@
     </row>
     <row r="44" spans="1:18">
       <c r="A44" s="19" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B44" s="19">
         <v>2021</v>
@@ -9368,7 +9368,7 @@
       </c>
       <c r="G44" s="13"/>
       <c r="H44" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I44" s="19">
         <v>2011</v>
@@ -9378,7 +9378,7 @@
       </c>
       <c r="O44" s="13"/>
       <c r="P44" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="Q44" s="19">
         <v>2011</v>
@@ -9389,7 +9389,7 @@
     </row>
     <row r="45" spans="1:18">
       <c r="A45" s="19" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B45" s="19">
         <v>2022</v>
@@ -9399,7 +9399,7 @@
       </c>
       <c r="G45" s="13"/>
       <c r="H45" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I45" s="19">
         <v>2012</v>
@@ -9409,7 +9409,7 @@
       </c>
       <c r="O45" s="13"/>
       <c r="P45" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="Q45" s="19">
         <v>2012</v>
@@ -9420,7 +9420,7 @@
     </row>
     <row r="46" spans="1:18">
       <c r="A46" s="19" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B46" s="19">
         <v>2023</v>
@@ -9430,7 +9430,7 @@
       </c>
       <c r="G46" s="13"/>
       <c r="H46" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I46" s="19">
         <v>2013</v>
@@ -9440,7 +9440,7 @@
       </c>
       <c r="O46" s="13"/>
       <c r="P46" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="Q46" s="19">
         <v>2013</v>
@@ -9451,7 +9451,7 @@
     </row>
     <row r="47" spans="1:18">
       <c r="A47" s="19" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B47" s="19">
         <v>2024</v>
@@ -9461,7 +9461,7 @@
       </c>
       <c r="G47" s="13"/>
       <c r="H47" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I47" s="19">
         <v>2014</v>
@@ -9471,7 +9471,7 @@
       </c>
       <c r="O47" s="13"/>
       <c r="P47" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="Q47" s="19">
         <v>2014</v>
@@ -9482,7 +9482,7 @@
     </row>
     <row r="48" spans="1:18">
       <c r="A48" s="19" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B48" s="19">
         <v>2025</v>
@@ -9492,7 +9492,7 @@
       </c>
       <c r="G48" s="13"/>
       <c r="H48" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I48" s="19">
         <v>2015</v>
@@ -9502,7 +9502,7 @@
       </c>
       <c r="O48" s="13"/>
       <c r="P48" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="Q48" s="19">
         <v>2015</v>
@@ -9514,7 +9514,7 @@
     <row r="49" spans="7:18">
       <c r="G49" s="13"/>
       <c r="H49" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I49" s="19">
         <v>2016</v>
@@ -9524,7 +9524,7 @@
       </c>
       <c r="O49" s="13"/>
       <c r="P49" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="Q49" s="19">
         <v>2016</v>
@@ -9536,7 +9536,7 @@
     <row r="50" spans="7:18">
       <c r="G50" s="13"/>
       <c r="H50" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I50" s="19">
         <v>2017</v>
@@ -9546,7 +9546,7 @@
       </c>
       <c r="O50" s="13"/>
       <c r="P50" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="Q50" s="19">
         <v>2017</v>
@@ -9558,7 +9558,7 @@
     <row r="51" spans="7:18">
       <c r="G51" s="13"/>
       <c r="H51" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I51" s="19">
         <v>2018</v>
@@ -9568,7 +9568,7 @@
       </c>
       <c r="O51" s="13"/>
       <c r="P51" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="Q51" s="19">
         <v>2018</v>
@@ -9580,7 +9580,7 @@
     <row r="52" spans="7:18">
       <c r="G52" s="13"/>
       <c r="H52" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I52" s="19">
         <v>2019</v>
@@ -9590,7 +9590,7 @@
       </c>
       <c r="O52" s="13"/>
       <c r="P52" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="Q52" s="19">
         <v>2019</v>
@@ -9602,7 +9602,7 @@
     <row r="53" spans="7:18">
       <c r="G53" s="13"/>
       <c r="H53" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I53" s="19">
         <v>2020</v>
@@ -9612,7 +9612,7 @@
       </c>
       <c r="O53" s="13"/>
       <c r="P53" s="19" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="Q53" s="19">
         <v>2020</v>
@@ -9624,7 +9624,7 @@
     <row r="54" spans="7:18">
       <c r="G54" s="13"/>
       <c r="H54" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I54" s="19">
         <v>2021</v>
@@ -9634,7 +9634,7 @@
       </c>
       <c r="O54" s="13"/>
       <c r="P54" s="19" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="Q54" s="19">
         <v>2021</v>
@@ -9646,7 +9646,7 @@
     <row r="55" spans="7:18">
       <c r="G55" s="13"/>
       <c r="H55" s="19" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="I55" s="19">
         <v>2022</v>
@@ -9656,7 +9656,7 @@
       </c>
       <c r="O55" s="13"/>
       <c r="P55" s="19" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="Q55" s="19">
         <v>2022</v>
@@ -9668,7 +9668,7 @@
     <row r="56" spans="7:18">
       <c r="G56" s="13"/>
       <c r="H56" s="19" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="I56" s="19">
         <v>2023</v>
@@ -9678,7 +9678,7 @@
       </c>
       <c r="O56" s="13"/>
       <c r="P56" s="19" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="Q56" s="19">
         <v>2023</v>
@@ -9690,7 +9690,7 @@
     <row r="57" spans="7:18">
       <c r="G57" s="13"/>
       <c r="H57" s="19" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="I57" s="19">
         <v>2024</v>
@@ -9700,7 +9700,7 @@
       </c>
       <c r="O57" s="13"/>
       <c r="P57" s="19" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="Q57" s="19">
         <v>2024</v>
@@ -9712,7 +9712,7 @@
     <row r="58" spans="7:18">
       <c r="G58" s="13"/>
       <c r="H58" s="19" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="I58" s="19">
         <v>2025</v>
@@ -9722,7 +9722,7 @@
       </c>
       <c r="O58" s="13"/>
       <c r="P58" s="19" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="Q58" s="19">
         <v>2025</v>

</xml_diff>